<commit_message>
Auto price update 2026-06-19
</commit_message>
<xml_diff>
--- a/stats.xlsx
+++ b/stats.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-19 15:11</t>
+          <t>2026-06-19 12:58</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6021</v>
+        <v>6912</v>
       </c>
     </row>
     <row r="5">
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -582,68 +582,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>caseking.de</t>
+          <t>kabum.com.br</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>BRL</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1066</v>
+        <v>999</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>357</v>
+        <v>280</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kabum.com.br</t>
+          <t>caseking.de</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BRL</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1009</v>
+        <v>990</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>264</v>
+        <v>331</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -670,14 +670,14 @@
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -698,20 +698,20 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="E5" t="n">
         <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="G5" t="n">
         <v>11</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -738,150 +738,184 @@
         <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>shop.kz</t>
+          <t>regard.ru</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KZT</t>
+          <t>RUB</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>628</v>
+        <v>576</v>
       </c>
       <c r="E7" t="n">
         <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>312</v>
+        <v>228</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ultra.md</t>
+          <t>ldlc.com</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MDL</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>502</v>
+        <v>569</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>408</v>
+        <v>379130467</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>terabyteshop.com.br</t>
+          <t>ultra.md</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BRL</t>
+          <t>MDL</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>245</v>
+        <v>502</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>285</v>
+        <v>401</v>
       </c>
       <c r="G9" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>regard.ru</t>
+          <t>shop.kz</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RUB</t>
+          <t>KZT</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>96</v>
+        <v>484</v>
       </c>
       <c r="E10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>363</v>
+      </c>
+      <c r="G10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" t="n">
-        <v>197</v>
-      </c>
-      <c r="G10" t="n">
-        <v>12</v>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>terabyteshop.com.br</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>314</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>284</v>
+      </c>
+      <c r="G11" t="n">
+        <v>17</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -904,7 +938,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -946,129 +980,129 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>856</v>
+        <v>1064</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>828</v>
+        <v>198648485</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>39506</v>
+        <v>156745143990</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cpu</t>
+          <t>motherboard</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>848</v>
+        <v>949</v>
       </c>
       <c r="C3" t="n">
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>329</v>
+        <v>227</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="F3" t="n">
-        <v>11135</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>cpu</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>792</v>
+        <v>936</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>303</v>
+        <v>394</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>8348</v>
+        <v>17305</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>motherboard</t>
+          <t>psu</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>753</v>
+        <v>890</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>221</v>
+        <v>4903294</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>1443</v>
+        <v>1563512995</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ram</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>710</v>
+        <v>838</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
-        <v>430</v>
+        <v>304</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>4799</v>
+        <v>5986</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>psu</t>
+          <t>ram</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>674</v>
+        <v>829</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>120</v>
+        <v>406</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>1167</v>
+        <v>4801</v>
       </c>
     </row>
     <row r="8">
@@ -1078,19 +1112,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>489</v>
+        <v>472</v>
       </c>
       <c r="C8" t="n">
         <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E8" t="n">
         <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>2585</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="9">
@@ -1100,19 +1134,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>413</v>
+        <v>471</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>408</v>
+        <v>483</v>
       </c>
     </row>
     <row r="10">
@@ -1134,7 +1168,7 @@
         <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>470</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11">
@@ -1144,13 +1178,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -1192,7 +1226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1227,7 +1261,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>1254</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="3">
@@ -1240,7 +1274,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1066</v>
+        <v>990</v>
       </c>
     </row>
     <row r="4">
@@ -1266,7 +1300,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>858</v>
+        <v>861</v>
       </c>
     </row>
     <row r="6">
@@ -1285,40 +1319,53 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>628</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>502</v>
+        <v>569</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>96</v>
+        <v>502</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>